<commit_message>
Fix amortization metadata label layout
</commit_message>
<xml_diff>
--- a/Project Rooms/Contract for Deed/transactions/320 Rose Pl - Ever Cardoza/output/320 Rose Pl - 12 Month Amortization Chart.xlsx
+++ b/Project Rooms/Contract for Deed/transactions/320 Rose Pl - Ever Cardoza/output/320 Rose Pl - 12 Month Amortization Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codex\Wiki Files\Project Rooms\Contract for Deed\transactions\320 Rose Pl - Ever Cardoza\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C053523-59CA-4D77-8232-1EE99E74446E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0B0D07-05A9-4A0F-A7E6-8B7DCE9FD598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{708B81A7-2176-43A6-9774-3105644AC06C}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>320 Rose Pl - 12 Month Amortization Chart</t>
   </si>
@@ -50,42 +50,12 @@
     <t>Buyer</t>
   </si>
   <si>
-    <t>Ever Cardoza / Maria Geraldina Sarmiento</t>
-  </si>
-  <si>
     <t>Property</t>
   </si>
   <si>
-    <t>320 Rose Pl</t>
-  </si>
-  <si>
-    <t>Contract date</t>
-  </si>
-  <si>
-    <t>7/1/2026</t>
-  </si>
-  <si>
-    <t>Sale amount</t>
-  </si>
-  <si>
-    <t>Down payment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20,790 </t>
-  </si>
-  <si>
-    <t>Loan amount</t>
-  </si>
-  <si>
     <t>Buyer rate</t>
   </si>
   <si>
-    <t>8.500%</t>
-  </si>
-  <si>
-    <t>Monthly total payment</t>
-  </si>
-  <si>
     <t>Payment #</t>
   </si>
   <si>
@@ -156,6 +126,21 @@
   </si>
   <si>
     <t>Totals for displayed 12-month period</t>
+  </si>
+  <si>
+    <t>Contract Date</t>
+  </si>
+  <si>
+    <t>Down Payment</t>
+  </si>
+  <si>
+    <t>Sale Amount</t>
+  </si>
+  <si>
+    <t>Loan Amount</t>
+  </si>
+  <si>
+    <t>Monthly Total Payment</t>
   </si>
 </sst>
 </file>
@@ -245,16 +230,8 @@
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -271,7 +248,19 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -613,753 +602,753 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="7" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="8.7109375" customWidth="1"/>
     <col min="8" max="9" width="10.7109375" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" customWidth="1"/>
     <col min="11" max="11" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="15"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="B6" s="15"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+    </row>
+    <row r="8" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="6" t="s">
+      <c r="D8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="7">
-        <v>346500</v>
-      </c>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="E8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="6" t="s">
+      <c r="G8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="7">
-        <v>325710</v>
-      </c>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="H8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="I8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="6" t="s">
+      <c r="J8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="7">
-        <v>2701</v>
-      </c>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-    </row>
-    <row r="8" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="K8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
+      <c r="A9" s="6">
         <f>1</f>
         <v>1</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="12">
+      <c r="B9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="8">
         <f>325710</f>
         <v>325710</v>
       </c>
-      <c r="D9" s="13">
-        <f>0.085</f>
+      <c r="D9" s="9">
+        <f t="shared" ref="D9:D20" si="0">0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E9" s="12">
-        <f>2504.43</f>
+      <c r="E9" s="8">
+        <f t="shared" ref="E9:E20" si="1">2504.43</f>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="8">
         <f>197.32</f>
         <v>197.32</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="8">
         <f>2307.11</f>
         <v>2307.11</v>
       </c>
-      <c r="H9" s="12">
-        <f>51.5</f>
+      <c r="H9" s="8">
+        <f t="shared" ref="H9:H20" si="2">51.5</f>
         <v>51.5</v>
       </c>
-      <c r="I9" s="12">
-        <f>145.096666666667</f>
+      <c r="I9" s="8">
+        <f t="shared" ref="I9:I20" si="3">145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
-      <c r="J9" s="12">
-        <f>2701.02666666667</f>
+      <c r="J9" s="8">
+        <f t="shared" ref="J9:J20" si="4">2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="8">
         <f>325512.68</f>
         <v>325512.68</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+      <c r="A10" s="6">
         <f>2</f>
         <v>2</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="12">
+      <c r="B10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="8">
         <f>325512.68</f>
         <v>325512.68</v>
       </c>
-      <c r="D10" s="13">
-        <f>0.085</f>
+      <c r="D10" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E10" s="12">
-        <f>2504.43</f>
+      <c r="E10" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="8">
         <f>198.72</f>
         <v>198.72</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="8">
         <f>2305.71</f>
         <v>2305.71</v>
       </c>
-      <c r="H10" s="12">
-        <f>51.5</f>
+      <c r="H10" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I10" s="12">
-        <f>145.096666666667</f>
+      <c r="I10" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J10" s="12">
-        <f>2701.02666666667</f>
+      <c r="J10" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="8">
         <f>325313.96</f>
         <v>325313.96000000002</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+      <c r="A11" s="6">
         <f>3</f>
         <v>3</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="12">
+      <c r="B11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="8">
         <f>325313.96</f>
         <v>325313.96000000002</v>
       </c>
-      <c r="D11" s="13">
-        <f>0.085</f>
+      <c r="D11" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E11" s="12">
-        <f>2504.43</f>
+      <c r="E11" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="8">
         <f>200.12</f>
         <v>200.12</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="8">
         <f>2304.31</f>
         <v>2304.31</v>
       </c>
-      <c r="H11" s="12">
-        <f>51.5</f>
+      <c r="H11" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I11" s="12">
-        <f>145.096666666667</f>
+      <c r="I11" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J11" s="12">
-        <f>2701.02666666667</f>
+      <c r="J11" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="8">
         <f>325113.84</f>
         <v>325113.84000000003</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="10">
+      <c r="A12" s="6">
         <f>4</f>
         <v>4</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="12">
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="8">
         <f>325113.84</f>
         <v>325113.84000000003</v>
       </c>
-      <c r="D12" s="13">
-        <f>0.085</f>
+      <c r="D12" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E12" s="12">
-        <f>2504.43</f>
+      <c r="E12" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="8">
         <f>201.54</f>
         <v>201.54</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="8">
         <f>2302.89</f>
         <v>2302.89</v>
       </c>
-      <c r="H12" s="12">
-        <f>51.5</f>
+      <c r="H12" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I12" s="12">
-        <f>145.096666666667</f>
+      <c r="I12" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J12" s="12">
-        <f>2701.02666666667</f>
+      <c r="J12" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K12" s="12">
+      <c r="K12" s="8">
         <f>324912.3</f>
         <v>324912.3</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="10">
+      <c r="A13" s="6">
         <f>5</f>
         <v>5</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="12">
+      <c r="B13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="8">
         <f>324912.3</f>
         <v>324912.3</v>
       </c>
-      <c r="D13" s="13">
-        <f>0.085</f>
+      <c r="D13" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E13" s="12">
-        <f>2504.43</f>
+      <c r="E13" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="8">
         <f>202.97</f>
         <v>202.97</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="8">
         <f>2301.46</f>
         <v>2301.46</v>
       </c>
-      <c r="H13" s="12">
-        <f>51.5</f>
+      <c r="H13" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I13" s="12">
-        <f>145.096666666667</f>
+      <c r="I13" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J13" s="12">
-        <f>2701.02666666667</f>
+      <c r="J13" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="8">
         <f>324709.33</f>
         <v>324709.33</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="10">
+      <c r="A14" s="6">
         <f>6</f>
         <v>6</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="12">
+      <c r="B14" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="8">
         <f>324709.33</f>
         <v>324709.33</v>
       </c>
-      <c r="D14" s="13">
-        <f>0.085</f>
+      <c r="D14" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E14" s="12">
-        <f>2504.43</f>
+      <c r="E14" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="8">
         <f>204.41</f>
         <v>204.41</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="8">
         <f>2300.02</f>
         <v>2300.02</v>
       </c>
-      <c r="H14" s="12">
-        <f>51.5</f>
+      <c r="H14" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I14" s="12">
-        <f>145.096666666667</f>
+      <c r="I14" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J14" s="12">
-        <f>2701.02666666667</f>
+      <c r="J14" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="8">
         <f>324504.92</f>
         <v>324504.92</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="10">
+      <c r="A15" s="6">
         <f>7</f>
         <v>7</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="12">
+      <c r="B15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="8">
         <f>324504.92</f>
         <v>324504.92</v>
       </c>
-      <c r="D15" s="13">
-        <f>0.085</f>
+      <c r="D15" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E15" s="12">
-        <f>2504.43</f>
+      <c r="E15" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="8">
         <f>205.85</f>
         <v>205.85</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="8">
         <f>2298.58</f>
         <v>2298.58</v>
       </c>
-      <c r="H15" s="12">
-        <f>51.5</f>
+      <c r="H15" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I15" s="12">
-        <f>145.096666666667</f>
+      <c r="I15" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J15" s="12">
-        <f>2701.02666666667</f>
+      <c r="J15" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="8">
         <f>324299.07</f>
         <v>324299.07</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="10">
+      <c r="A16" s="6">
         <f>8</f>
         <v>8</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="12">
+      <c r="B16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="8">
         <f>324299.07</f>
         <v>324299.07</v>
       </c>
-      <c r="D16" s="13">
-        <f>0.085</f>
+      <c r="D16" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E16" s="12">
-        <f>2504.43</f>
+      <c r="E16" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="8">
         <f>207.31</f>
         <v>207.31</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="8">
         <f>2297.12</f>
         <v>2297.12</v>
       </c>
-      <c r="H16" s="12">
-        <f>51.5</f>
+      <c r="H16" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I16" s="12">
-        <f>145.096666666667</f>
+      <c r="I16" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J16" s="12">
-        <f>2701.02666666667</f>
+      <c r="J16" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K16" s="12">
+      <c r="K16" s="8">
         <f>324091.76</f>
         <v>324091.76</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="10">
+      <c r="A17" s="6">
         <f>9</f>
         <v>9</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="12">
+      <c r="B17" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="8">
         <f>324091.76</f>
         <v>324091.76</v>
       </c>
-      <c r="D17" s="13">
-        <f>0.085</f>
+      <c r="D17" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E17" s="12">
-        <f>2504.43</f>
+      <c r="E17" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="8">
         <f>208.78</f>
         <v>208.78</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="8">
         <f>2295.65</f>
         <v>2295.65</v>
       </c>
-      <c r="H17" s="12">
-        <f>51.5</f>
+      <c r="H17" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I17" s="12">
-        <f>145.096666666667</f>
+      <c r="I17" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J17" s="12">
-        <f>2701.02666666667</f>
+      <c r="J17" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K17" s="12">
+      <c r="K17" s="8">
         <f>323882.98</f>
         <v>323882.98</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="10">
+      <c r="A18" s="6">
         <f>10</f>
         <v>10</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="12">
+      <c r="B18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="8">
         <f>323882.98</f>
         <v>323882.98</v>
       </c>
-      <c r="D18" s="13">
-        <f>0.085</f>
+      <c r="D18" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E18" s="12">
-        <f>2504.43</f>
+      <c r="E18" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="8">
         <f>210.26</f>
         <v>210.26</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="8">
         <f>2294.17</f>
         <v>2294.17</v>
       </c>
-      <c r="H18" s="12">
-        <f>51.5</f>
+      <c r="H18" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I18" s="12">
-        <f>145.096666666667</f>
+      <c r="I18" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J18" s="12">
-        <f>2701.02666666667</f>
+      <c r="J18" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K18" s="12">
+      <c r="K18" s="8">
         <f>323672.72</f>
         <v>323672.71999999997</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="10">
+      <c r="A19" s="6">
         <f>11</f>
         <v>11</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="12">
+      <c r="B19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="8">
         <f>323672.72</f>
         <v>323672.71999999997</v>
       </c>
-      <c r="D19" s="13">
-        <f>0.085</f>
+      <c r="D19" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E19" s="12">
-        <f>2504.43</f>
+      <c r="E19" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="8">
         <f>211.75</f>
         <v>211.75</v>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="8">
         <f>2292.68</f>
         <v>2292.6799999999998</v>
       </c>
-      <c r="H19" s="12">
-        <f>51.5</f>
+      <c r="H19" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I19" s="12">
-        <f>145.096666666667</f>
+      <c r="I19" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J19" s="12">
-        <f>2701.02666666667</f>
+      <c r="J19" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K19" s="12">
+      <c r="K19" s="8">
         <f>323460.97</f>
         <v>323460.96999999997</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="10">
+      <c r="A20" s="6">
         <f>12</f>
         <v>12</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="12">
+      <c r="B20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="8">
         <f>323460.97</f>
         <v>323460.96999999997</v>
       </c>
-      <c r="D20" s="13">
-        <f>0.085</f>
+      <c r="D20" s="9">
+        <f t="shared" si="0"/>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E20" s="12">
-        <f>2504.43</f>
+      <c r="E20" s="8">
+        <f t="shared" si="1"/>
         <v>2504.4299999999998</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="8">
         <f>213.25</f>
         <v>213.25</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="8">
         <f>2291.18</f>
         <v>2291.1799999999998</v>
       </c>
-      <c r="H20" s="12">
-        <f>51.5</f>
+      <c r="H20" s="8">
+        <f t="shared" si="2"/>
         <v>51.5</v>
       </c>
-      <c r="I20" s="12">
-        <f>145.096666666667</f>
+      <c r="I20" s="8">
+        <f t="shared" si="3"/>
         <v>145.09666666666701</v>
       </c>
-      <c r="J20" s="12">
-        <f>2701.02666666667</f>
+      <c r="J20" s="8">
+        <f t="shared" si="4"/>
         <v>2701.0266666666698</v>
       </c>
-      <c r="K20" s="12">
+      <c r="K20" s="8">
         <f>323247.72</f>
         <v>323247.71999999997</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
-      <c r="E21" s="15">
-        <f>SUM(E9:E20)</f>
+      <c r="E21" s="11">
+        <f t="shared" ref="E21:J21" si="5">SUM(E9:E20)</f>
         <v>30053.16</v>
       </c>
-      <c r="F21" s="15">
-        <f>SUM(F9:F20)</f>
+      <c r="F21" s="11">
+        <f t="shared" si="5"/>
         <v>2462.2799999999997</v>
       </c>
-      <c r="G21" s="15">
-        <f>SUM(G9:G20)</f>
+      <c r="G21" s="11">
+        <f t="shared" si="5"/>
         <v>27590.880000000005</v>
       </c>
-      <c r="H21" s="15">
-        <f>SUM(H9:H20)</f>
+      <c r="H21" s="11">
+        <f t="shared" si="5"/>
         <v>618</v>
       </c>
-      <c r="I21" s="15">
-        <f>SUM(I9:I20)</f>
+      <c r="I21" s="11">
+        <f t="shared" si="5"/>
         <v>1741.1600000000042</v>
       </c>
-      <c r="J21" s="15">
-        <f>SUM(J9:J20)</f>
+      <c r="J21" s="11">
+        <f t="shared" si="5"/>
         <v>32412.320000000032</v>
       </c>
-      <c r="K21" s="16"/>
+      <c r="K21" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="18">
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:K3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:E6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4800" verticalDpi="4800" r:id="rId1"/>

</xml_diff>

<commit_message>
Add amortization chart template workflow
</commit_message>
<xml_diff>
--- a/Project Rooms/Contract for Deed/transactions/320 Rose Pl - Ever Cardoza/output/320 Rose Pl - 12 Month Amortization Chart.xlsx
+++ b/Project Rooms/Contract for Deed/transactions/320 Rose Pl - Ever Cardoza/output/320 Rose Pl - 12 Month Amortization Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codex\Wiki Files\Project Rooms\Contract for Deed\transactions\320 Rose Pl - Ever Cardoza\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0B0D07-05A9-4A0F-A7E6-8B7DCE9FD598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63DD9AB-4F41-4A64-A8C1-341C3CE035DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{708B81A7-2176-43A6-9774-3105644AC06C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{06CA6E75-7099-4174-99F2-A983CB5A5C31}"/>
   </bookViews>
   <sheets>
     <sheet name="12 Month Chart" sheetId="1" r:id="rId1"/>
@@ -42,51 +42,75 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+  <si>
+    <t>Buyer</t>
+  </si>
+  <si>
+    <t>Property</t>
+  </si>
+  <si>
+    <t>Contract Date</t>
+  </si>
+  <si>
+    <t>Sale Amount</t>
+  </si>
+  <si>
+    <t>Down Payment</t>
+  </si>
+  <si>
+    <t>Loan Amount</t>
+  </si>
+  <si>
+    <t>Buyer Rate</t>
+  </si>
+  <si>
+    <t>Monthly Total Payment</t>
+  </si>
+  <si>
+    <t>Payment #</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Beginning Balance</t>
+  </si>
+  <si>
+    <t>Interest Rate</t>
+  </si>
+  <si>
+    <t>Scheduled Payment</t>
+  </si>
+  <si>
+    <t>Principal</t>
+  </si>
+  <si>
+    <t>Interest</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Taxes</t>
+  </si>
+  <si>
+    <t>Total Payment</t>
+  </si>
+  <si>
+    <t>Ending Balance</t>
+  </si>
+  <si>
+    <t>Totals for displayed 12-month period</t>
+  </si>
   <si>
     <t>320 Rose Pl - 12 Month Amortization Chart</t>
   </si>
   <si>
-    <t>Buyer</t>
-  </si>
-  <si>
-    <t>Property</t>
-  </si>
-  <si>
-    <t>Buyer rate</t>
-  </si>
-  <si>
-    <t>Payment #</t>
-  </si>
-  <si>
-    <t>Due Date</t>
-  </si>
-  <si>
-    <t>Beginning Balance</t>
-  </si>
-  <si>
-    <t>Interest Rate</t>
-  </si>
-  <si>
-    <t>Scheduled Payment</t>
-  </si>
-  <si>
-    <t>Principal</t>
-  </si>
-  <si>
-    <t>Interest</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Taxes</t>
-  </si>
-  <si>
-    <t>Total Payment</t>
-  </si>
-  <si>
-    <t>Ending Balance</t>
+    <t>Ever Cardoza / Maria Geraldina Sarmiento</t>
+  </si>
+  <si>
+    <t>320 Rose Pl</t>
   </si>
   <si>
     <t>Jul-26</t>
@@ -123,24 +147,6 @@
   </si>
   <si>
     <t>Jun-27</t>
-  </si>
-  <si>
-    <t>Totals for displayed 12-month period</t>
-  </si>
-  <si>
-    <t>Contract Date</t>
-  </si>
-  <si>
-    <t>Down Payment</t>
-  </si>
-  <si>
-    <t>Sale Amount</t>
-  </si>
-  <si>
-    <t>Loan Amount</t>
-  </si>
-  <si>
-    <t>Monthly Total Payment</t>
   </si>
 </sst>
 </file>
@@ -227,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -248,17 +254,26 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -594,7 +609,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40547C1B-7023-4DD8-9CDA-B68232D3B795}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88EC3160-80CC-4353-B980-C42AFE243717}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -603,29 +618,25 @@
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="7" width="8.7109375" customWidth="1"/>
-    <col min="8" max="9" width="10.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="3" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
+      <c r="A1" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -641,72 +652,88 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="14"/>
+      <c r="H3" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="17">
+        <v>46204</v>
+      </c>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="18">
+        <v>346500</v>
+      </c>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
+      <c r="A5" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="18">
+        <v>20790</v>
+      </c>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="14"/>
+      <c r="H5" s="18">
+        <v>325710</v>
+      </c>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
+      <c r="A6" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="19">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="18">
+        <v>2701</v>
+      </c>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -723,37 +750,37 @@
     </row>
     <row r="8" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -762,18 +789,18 @@
         <v>1</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C9" s="8">
         <f>325710</f>
         <v>325710</v>
       </c>
       <c r="D9" s="9">
-        <f t="shared" ref="D9:D20" si="0">0.085</f>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E9" s="8">
-        <f t="shared" ref="E9:E20" si="1">2504.43</f>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F9" s="8">
@@ -785,15 +812,15 @@
         <v>2307.11</v>
       </c>
       <c r="H9" s="8">
-        <f t="shared" ref="H9:H20" si="2">51.5</f>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I9" s="8">
-        <f t="shared" ref="I9:I20" si="3">145.096666666667</f>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J9" s="8">
-        <f t="shared" ref="J9:J20" si="4">2701.02666666667</f>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K9" s="8">
@@ -807,18 +834,18 @@
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C10" s="8">
         <f>325512.68</f>
         <v>325512.68</v>
       </c>
       <c r="D10" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E10" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F10" s="8">
@@ -830,15 +857,15 @@
         <v>2305.71</v>
       </c>
       <c r="H10" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I10" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J10" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K10" s="8">
@@ -852,18 +879,18 @@
         <v>3</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C11" s="8">
         <f>325313.96</f>
         <v>325313.96000000002</v>
       </c>
       <c r="D11" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E11" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F11" s="8">
@@ -875,15 +902,15 @@
         <v>2304.31</v>
       </c>
       <c r="H11" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I11" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J11" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K11" s="8">
@@ -897,18 +924,18 @@
         <v>4</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C12" s="8">
         <f>325113.84</f>
         <v>325113.84000000003</v>
       </c>
       <c r="D12" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E12" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F12" s="8">
@@ -920,15 +947,15 @@
         <v>2302.89</v>
       </c>
       <c r="H12" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I12" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J12" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K12" s="8">
@@ -942,18 +969,18 @@
         <v>5</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C13" s="8">
         <f>324912.3</f>
         <v>324912.3</v>
       </c>
       <c r="D13" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E13" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F13" s="8">
@@ -965,15 +992,15 @@
         <v>2301.46</v>
       </c>
       <c r="H13" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I13" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J13" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K13" s="8">
@@ -987,18 +1014,18 @@
         <v>6</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C14" s="8">
         <f>324709.33</f>
         <v>324709.33</v>
       </c>
       <c r="D14" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E14" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F14" s="8">
@@ -1010,15 +1037,15 @@
         <v>2300.02</v>
       </c>
       <c r="H14" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I14" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J14" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K14" s="8">
@@ -1032,18 +1059,18 @@
         <v>7</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C15" s="8">
         <f>324504.92</f>
         <v>324504.92</v>
       </c>
       <c r="D15" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E15" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F15" s="8">
@@ -1055,15 +1082,15 @@
         <v>2298.58</v>
       </c>
       <c r="H15" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I15" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J15" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K15" s="8">
@@ -1077,18 +1104,18 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C16" s="8">
         <f>324299.07</f>
         <v>324299.07</v>
       </c>
       <c r="D16" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E16" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F16" s="8">
@@ -1100,15 +1127,15 @@
         <v>2297.12</v>
       </c>
       <c r="H16" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I16" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J16" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K16" s="8">
@@ -1122,18 +1149,18 @@
         <v>9</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C17" s="8">
         <f>324091.76</f>
         <v>324091.76</v>
       </c>
       <c r="D17" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E17" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F17" s="8">
@@ -1145,15 +1172,15 @@
         <v>2295.65</v>
       </c>
       <c r="H17" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I17" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J17" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K17" s="8">
@@ -1167,18 +1194,18 @@
         <v>10</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C18" s="8">
         <f>323882.98</f>
         <v>323882.98</v>
       </c>
       <c r="D18" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E18" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F18" s="8">
@@ -1190,15 +1217,15 @@
         <v>2294.17</v>
       </c>
       <c r="H18" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I18" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J18" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K18" s="8">
@@ -1212,18 +1239,18 @@
         <v>11</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C19" s="8">
         <f>323672.72</f>
         <v>323672.71999999997</v>
       </c>
       <c r="D19" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E19" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F19" s="8">
@@ -1235,15 +1262,15 @@
         <v>2292.6799999999998</v>
       </c>
       <c r="H19" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I19" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J19" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K19" s="8">
@@ -1257,18 +1284,18 @@
         <v>12</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C20" s="8">
         <f>323460.97</f>
         <v>323460.96999999997</v>
       </c>
       <c r="D20" s="9">
-        <f t="shared" si="0"/>
+        <f>0.085</f>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="E20" s="8">
-        <f t="shared" si="1"/>
+        <f>2504.43</f>
         <v>2504.4299999999998</v>
       </c>
       <c r="F20" s="8">
@@ -1280,15 +1307,15 @@
         <v>2291.1799999999998</v>
       </c>
       <c r="H20" s="8">
-        <f t="shared" si="2"/>
+        <f>51.5</f>
         <v>51.5</v>
       </c>
       <c r="I20" s="8">
-        <f t="shared" si="3"/>
+        <f>145.096666666667</f>
         <v>145.09666666666701</v>
       </c>
       <c r="J20" s="8">
-        <f t="shared" si="4"/>
+        <f>2701.02666666667</f>
         <v>2701.0266666666698</v>
       </c>
       <c r="K20" s="8">
@@ -1297,58 +1324,58 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
+      <c r="A21" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
       <c r="E21" s="11">
-        <f t="shared" ref="E21:J21" si="5">SUM(E9:E20)</f>
+        <f t="shared" ref="E21:J21" si="0">SUM(E9:E20)</f>
         <v>30053.16</v>
       </c>
       <c r="F21" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v>2462.2799999999997</v>
       </c>
       <c r="G21" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v>27590.880000000005</v>
       </c>
       <c r="H21" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v>618</v>
       </c>
       <c r="I21" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v>1741.1600000000042</v>
       </c>
       <c r="J21" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="0"/>
         <v>32412.320000000032</v>
       </c>
       <c r="K21" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:K4"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="H3:K3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="H5:K5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:K6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4800" verticalDpi="4800" r:id="rId1"/>

</xml_diff>